<commit_message>
correcciones mostrar las IEs, mostrar las iamgenes y archivos que se envian, correccion de plantilla
</commit_message>
<xml_diff>
--- a/public/plantillas/PlantillaCargueEstudiantes.xlsx
+++ b/public/plantillas/PlantillaCargueEstudiantes.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Personal\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kian1\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B11652D-C70E-4509-B66D-090FCC7BD54D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AEF6BB-486E-4427-A212-1FFEC22222C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="10620" windowHeight="10428" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="proc9319259" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">proc9319259!$Q$2:$Q$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">proc9319259!$Q$1:$Q$1</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>SEDE</t>
   </si>
@@ -101,71 +101,59 @@
     <t>TIPO_DE_SANGRE</t>
   </si>
   <si>
-    <t>Columna1</t>
-  </si>
-  <si>
-    <t>Columna2</t>
-  </si>
-  <si>
-    <t>Columna3</t>
-  </si>
-  <si>
-    <t>Columna4</t>
-  </si>
-  <si>
-    <t>Columna5</t>
-  </si>
-  <si>
-    <t>Columna6</t>
-  </si>
-  <si>
-    <t>Columna7</t>
-  </si>
-  <si>
-    <t>Columna8</t>
-  </si>
-  <si>
-    <t>Columna9</t>
-  </si>
-  <si>
-    <t>Columna10</t>
-  </si>
-  <si>
-    <t>Columna11</t>
-  </si>
-  <si>
-    <t>Columna12</t>
-  </si>
-  <si>
-    <t>Columna13</t>
-  </si>
-  <si>
-    <t>Columna14</t>
-  </si>
-  <si>
-    <t>Columna15</t>
-  </si>
-  <si>
-    <t>Columna16</t>
-  </si>
-  <si>
-    <t>Columna17</t>
-  </si>
-  <si>
-    <t>Columna18</t>
-  </si>
-  <si>
-    <t>Columna19</t>
-  </si>
-  <si>
-    <t>Columna20</t>
+    <t>ÚNICA</t>
+  </si>
+  <si>
+    <t>ESTRATO 1</t>
+  </si>
+  <si>
+    <t>B1</t>
+  </si>
+  <si>
+    <t>TI:TARJETA DE IDENTIDAD</t>
+  </si>
+  <si>
+    <t>MASCULINO</t>
+  </si>
+  <si>
+    <t>O +</t>
+  </si>
+  <si>
+    <t>NO APLICA</t>
+  </si>
+  <si>
+    <t>COLOMBIA</t>
+  </si>
+  <si>
+    <t>SILVANIA</t>
+  </si>
+  <si>
+    <t>NUEVA EPS</t>
+  </si>
+  <si>
+    <t>BRISAS</t>
+  </si>
+  <si>
+    <t>CORREO@EXAMPLE.COM</t>
+  </si>
+  <si>
+    <t>JHON</t>
+  </si>
+  <si>
+    <t>ALEX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESPAÑA </t>
+  </si>
+  <si>
+    <t>RODRIGUEZ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -296,6 +284,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -598,7 +594,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -641,11 +637,15 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Énfasis2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Énfasis3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -677,6 +677,7 @@
     <cellStyle name="Énfasis5" xfId="34" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Énfasis6" xfId="38" builtinId="49" customBuiltin="1"/>
     <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Hipervínculo" xfId="42" builtinId="8"/>
     <cellStyle name="Incorrecto" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -706,26 +707,26 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A93AC754-A211-49BA-B85C-434BCCD8F0D2}" name="Tabla1" displayName="Tabla1" ref="A1:T25" totalsRowShown="0">
   <autoFilter ref="A1:T25" xr:uid="{A93AC754-A211-49BA-B85C-434BCCD8F0D2}"/>
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{5E23EBC9-3F97-4B68-A9BF-2DDA0CEB7A1E}" name="Columna1"/>
-    <tableColumn id="2" xr3:uid="{A4F157D1-4DCD-4FCE-AEF6-D23016FBC97D}" name="Columna2"/>
-    <tableColumn id="3" xr3:uid="{BC8E24E1-1AA9-4C28-BA09-6C577B706614}" name="Columna3"/>
-    <tableColumn id="4" xr3:uid="{86A16690-80AD-4304-BD62-EDA419FD63BA}" name="Columna4"/>
-    <tableColumn id="5" xr3:uid="{67FBFEA3-A629-4DFF-92CF-EC984B6F68CB}" name="Columna5"/>
-    <tableColumn id="6" xr3:uid="{36DB76EE-5BFF-4BE3-90B2-7CDE6CB9F236}" name="Columna6"/>
-    <tableColumn id="7" xr3:uid="{1E41998A-BD75-41E0-B90E-A8AE9B3F67F3}" name="Columna7"/>
-    <tableColumn id="8" xr3:uid="{FFBE1F65-904D-4F22-A814-8C8B3A65EAB9}" name="Columna8"/>
-    <tableColumn id="9" xr3:uid="{0053D8BC-9B89-41FD-8277-565E9A431985}" name="Columna9"/>
-    <tableColumn id="10" xr3:uid="{63020D04-9CC7-4CF0-9514-B8504E98F523}" name="Columna10"/>
-    <tableColumn id="11" xr3:uid="{BAEC058C-04E5-4905-9353-2A4F7176B01E}" name="Columna11"/>
-    <tableColumn id="12" xr3:uid="{BA020A8E-E3AD-4329-A365-40E10ACC08DD}" name="Columna12"/>
-    <tableColumn id="13" xr3:uid="{8A68BC7E-6957-4631-BA08-0BB5354E5A38}" name="Columna13"/>
-    <tableColumn id="14" xr3:uid="{26F3DBAA-3957-4C99-8031-7BFB740993B3}" name="Columna14"/>
-    <tableColumn id="15" xr3:uid="{4F51E9C4-9C35-4AFA-92DB-F4216C98F62F}" name="Columna15"/>
-    <tableColumn id="16" xr3:uid="{76C85BCB-B199-4C21-B2FE-285AD9DA831F}" name="Columna16"/>
-    <tableColumn id="17" xr3:uid="{CABB1548-B117-4682-9313-C0F431EBE61D}" name="Columna17"/>
-    <tableColumn id="18" xr3:uid="{072B1EAE-F8A1-4602-AF0B-DCD647B5F3DB}" name="Columna18"/>
-    <tableColumn id="19" xr3:uid="{85BF805D-78C9-44CC-8184-54CD589F962F}" name="Columna19"/>
-    <tableColumn id="20" xr3:uid="{8B8DD314-0298-4AB9-8E68-E1CFDFE2EDBA}" name="Columna20"/>
+    <tableColumn id="1" xr3:uid="{5E23EBC9-3F97-4B68-A9BF-2DDA0CEB7A1E}" name="SEDE"/>
+    <tableColumn id="2" xr3:uid="{A4F157D1-4DCD-4FCE-AEF6-D23016FBC97D}" name="JORNADA"/>
+    <tableColumn id="3" xr3:uid="{BC8E24E1-1AA9-4C28-BA09-6C577B706614}" name="FECHAINI"/>
+    <tableColumn id="4" xr3:uid="{86A16690-80AD-4304-BD62-EDA419FD63BA}" name="ESTRATO"/>
+    <tableColumn id="5" xr3:uid="{67FBFEA3-A629-4DFF-92CF-EC984B6F68CB}" name="SISBEN_IV"/>
+    <tableColumn id="6" xr3:uid="{36DB76EE-5BFF-4BE3-90B2-7CDE6CB9F236}" name="DOC"/>
+    <tableColumn id="7" xr3:uid="{1E41998A-BD75-41E0-B90E-A8AE9B3F67F3}" name="TIPODOC"/>
+    <tableColumn id="8" xr3:uid="{FFBE1F65-904D-4F22-A814-8C8B3A65EAB9}" name="APELLIDO1"/>
+    <tableColumn id="9" xr3:uid="{0053D8BC-9B89-41FD-8277-565E9A431985}" name="APELLIDO2"/>
+    <tableColumn id="10" xr3:uid="{63020D04-9CC7-4CF0-9514-B8504E98F523}" name="NOMBRE1"/>
+    <tableColumn id="11" xr3:uid="{BAEC058C-04E5-4905-9353-2A4F7176B01E}" name="NOMBRE2"/>
+    <tableColumn id="12" xr3:uid="{BA020A8E-E3AD-4329-A365-40E10ACC08DD}" name="GENERO"/>
+    <tableColumn id="13" xr3:uid="{8A68BC7E-6957-4631-BA08-0BB5354E5A38}" name="FECHA_NACIMIENTO"/>
+    <tableColumn id="14" xr3:uid="{26F3DBAA-3957-4C99-8031-7BFB740993B3}" name="BARRIO"/>
+    <tableColumn id="15" xr3:uid="{4F51E9C4-9C35-4AFA-92DB-F4216C98F62F}" name="EPS"/>
+    <tableColumn id="16" xr3:uid="{76C85BCB-B199-4C21-B2FE-285AD9DA831F}" name="TIPO_DE_SANGRE"/>
+    <tableColumn id="17" xr3:uid="{CABB1548-B117-4682-9313-C0F431EBE61D}" name="DISCAPACIDAD"/>
+    <tableColumn id="18" xr3:uid="{072B1EAE-F8A1-4602-AF0B-DCD647B5F3DB}" name="PAIS_ORIGEN"/>
+    <tableColumn id="19" xr3:uid="{85BF805D-78C9-44CC-8184-54CD589F962F}" name="CORREO"/>
+    <tableColumn id="20" xr3:uid="{8B8DD314-0298-4AB9-8E68-E1CFDFE2EDBA}" name="TELEFONO"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1028,151 +1029,187 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:T9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.109375" customWidth="1"/>
     <col min="4" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" customWidth="1"/>
+    <col min="8" max="8" width="11.5546875" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
     <col min="10" max="12" width="13" customWidth="1"/>
-    <col min="13" max="13" width="22.42578125" customWidth="1"/>
+    <col min="13" max="13" width="22.44140625" customWidth="1"/>
     <col min="14" max="15" width="13" customWidth="1"/>
-    <col min="16" max="16" width="18.42578125" customWidth="1"/>
-    <col min="17" max="17" width="17.85546875" customWidth="1"/>
-    <col min="18" max="18" width="14.7109375" customWidth="1"/>
+    <col min="16" max="16" width="18.44140625" customWidth="1"/>
+    <col min="17" max="17" width="17.88671875" customWidth="1"/>
+    <col min="18" max="18" width="14.6640625" customWidth="1"/>
     <col min="19" max="20" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>14</v>
+      </c>
+      <c r="R1" t="s">
+        <v>15</v>
+      </c>
+      <c r="S1" t="s">
+        <v>16</v>
+      </c>
+      <c r="T1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" t="s">
         <v>20</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C2" s="1">
+        <v>45993.847002314818</v>
+      </c>
+      <c r="D2" t="s">
         <v>21</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E2" t="s">
         <v>22</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F2">
+        <v>1077200000</v>
+      </c>
+      <c r="G2" t="s">
         <v>23</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J2" t="s">
+        <v>32</v>
+      </c>
+      <c r="K2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L2" t="s">
         <v>24</v>
       </c>
-      <c r="F1" t="s">
+      <c r="M2" s="2">
+        <v>42663</v>
+      </c>
+      <c r="N2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O2" t="s">
+        <v>29</v>
+      </c>
+      <c r="P2" t="s">
         <v>25</v>
       </c>
-      <c r="G1" t="s">
+      <c r="Q2" t="s">
         <v>26</v>
       </c>
-      <c r="H1" t="s">
+      <c r="R2" t="s">
         <v>27</v>
       </c>
-      <c r="I1" t="s">
-        <v>28</v>
-      </c>
-      <c r="J1" t="s">
-        <v>29</v>
-      </c>
-      <c r="K1" t="s">
-        <v>30</v>
-      </c>
-      <c r="L1" t="s">
+      <c r="S2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="M1" t="s">
-        <v>32</v>
-      </c>
-      <c r="N1" t="s">
-        <v>33</v>
-      </c>
-      <c r="O1" t="s">
-        <v>34</v>
-      </c>
-      <c r="P1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>36</v>
-      </c>
-      <c r="R1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S1" t="s">
-        <v>38</v>
-      </c>
-      <c r="T1" t="s">
-        <v>39</v>
+      <c r="T2">
+        <v>3224019127</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" t="s">
-        <v>6</v>
-      </c>
-      <c r="I2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J2" t="s">
-        <v>8</v>
-      </c>
-      <c r="K2" t="s">
-        <v>9</v>
-      </c>
-      <c r="L2" t="s">
-        <v>10</v>
-      </c>
-      <c r="M2" t="s">
-        <v>11</v>
-      </c>
-      <c r="N2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O2" t="s">
-        <v>13</v>
-      </c>
-      <c r="P2" t="s">
-        <v>19</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>14</v>
-      </c>
-      <c r="R2" t="s">
-        <v>15</v>
-      </c>
-      <c r="S2" t="s">
-        <v>16</v>
-      </c>
-      <c r="T2" t="s">
-        <v>17</v>
-      </c>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="C3" s="1"/>
+      <c r="M3" s="2"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="C4" s="1"/>
+      <c r="M4" s="2"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="C5" s="1"/>
+      <c r="M5" s="2"/>
+      <c r="S5" s="3"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="C6" s="1"/>
+      <c r="M6" s="2"/>
+      <c r="S6" s="3"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="C7" s="1"/>
+      <c r="M7" s="2"/>
+      <c r="S7" s="3"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="C8" s="1"/>
+      <c r="M8" s="2"/>
+      <c r="S8" s="3"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="C9" s="1"/>
+      <c r="M9" s="2"/>
+      <c r="S9" s="3"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="S2" r:id="rId1" xr:uid="{3FE075D1-5ED0-4F3B-8473-CD70793588EB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>